<commit_message>
Dashboard 2026-09-22 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/341101559/spec-341101559.xlsx
+++ b/vse-loti/341101559/spec-341101559.xlsx
@@ -1709,16 +1709,16 @@
         </is>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.155</v>
+        <v>1.282</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>281000</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>1812903.23</v>
+        <v>219188.77</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>2211741.94</v>
+        <v>267410.3</v>
       </c>
     </row>
     <row r="43">
@@ -1744,16 +1744,16 @@
         </is>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.186</v>
+        <v>1.539</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>337200</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>1812903.23</v>
+        <v>219103.31</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>2211741.94</v>
+        <v>267306.04</v>
       </c>
     </row>
     <row r="44">
@@ -1779,16 +1779,16 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.257</v>
+        <v>2.127</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>362863.68</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>1411920.93</v>
+        <v>170598.82</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>1722543.54</v>
+        <v>208130.55</v>
       </c>
     </row>
     <row r="45">
@@ -1814,16 +1814,16 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.311</v>
+        <v>2.572</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>438948</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>1411408.36</v>
+        <v>170664.07</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>1721918.2</v>
+        <v>208210.17</v>
       </c>
     </row>
     <row r="46">
@@ -1849,16 +1849,16 @@
         </is>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.381</v>
+        <v>3.152</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>646187</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>1696028.87</v>
+        <v>205008.57</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>2069155.22</v>
+        <v>250110.45</v>
       </c>
     </row>
     <row r="47">
@@ -1884,16 +1884,16 @@
         </is>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.556</v>
+        <v>4.592</v>
       </c>
       <c r="G47" s="4" t="n">
         <v>887940</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>1597014.39</v>
+        <v>193366.72</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>1948357.55</v>
+        <v>235907.4</v>
       </c>
     </row>
     <row r="48">
@@ -1919,16 +1919,16 @@
         </is>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1.329</v>
+        <v>10.98</v>
       </c>
       <c r="G48" s="4" t="n">
         <v>1297108</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>976003.01</v>
+        <v>118133.7</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>1190723.67</v>
+        <v>144123.11</v>
       </c>
     </row>
     <row r="49">
@@ -1954,16 +1954,16 @@
         </is>
       </c>
       <c r="F49" s="5" t="n">
-        <v>2.495</v>
+        <v>20.614</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>4486119.45</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>1798043.87</v>
+        <v>217624.89</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>2193613.52</v>
+        <v>265502.36</v>
       </c>
     </row>
     <row r="50">
@@ -1989,16 +1989,16 @@
         </is>
       </c>
       <c r="F50" s="5" t="n">
-        <v>1.313</v>
+        <v>10.85</v>
       </c>
       <c r="G50" s="4" t="n">
         <v>2361115.5</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>1798260.09</v>
+        <v>217614.33</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>2193877.31</v>
+        <v>265489.48</v>
       </c>
     </row>
     <row r="51">
@@ -2024,16 +2024,16 @@
         </is>
       </c>
       <c r="F51" s="5" t="n">
-        <v>3.116</v>
+        <v>25.747</v>
       </c>
       <c r="G51" s="4" t="n">
         <v>6748672.5</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>2165812.74</v>
+        <v>262114.91</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>2642291.54</v>
+        <v>319780.19</v>
       </c>
     </row>
     <row r="52">
@@ -2059,16 +2059,16 @@
         </is>
       </c>
       <c r="F52" s="5" t="n">
-        <v>3.739</v>
+        <v>30.897</v>
       </c>
       <c r="G52" s="4" t="n">
         <v>8098407</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>2165928.59</v>
+        <v>262109.82</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>2642432.88</v>
+        <v>319773.98</v>
       </c>
     </row>
     <row r="53">
@@ -2094,16 +2094,16 @@
         </is>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.056</v>
+        <v>0.462</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>128067</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>2286910.71</v>
+        <v>277201.3</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>2790031.07</v>
+        <v>338185.58</v>
       </c>
     </row>
     <row r="54">
@@ -2129,16 +2129,16 @@
         </is>
       </c>
       <c r="F54" s="5" t="n">
-        <v>11.129</v>
+        <v>91.96599999999999</v>
       </c>
       <c r="G54" s="4" t="n">
         <v>25010378.18</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>2247315.86</v>
+        <v>271952.44</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>2741725.35</v>
+        <v>331781.98</v>
       </c>
     </row>
     <row r="55">
@@ -2164,16 +2164,16 @@
         </is>
       </c>
       <c r="F55" s="5" t="n">
-        <v>4.455</v>
+        <v>36.816</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>10012161</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>2247398.65</v>
+        <v>271951.35</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>2741826.36</v>
+        <v>331780.65</v>
       </c>
     </row>
     <row r="56">
@@ -2199,16 +2199,16 @@
         </is>
       </c>
       <c r="F56" s="5" t="n">
-        <v>7.242</v>
+        <v>59.857</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>16382058.1</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>2262090.32</v>
+        <v>273686.59</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>2759750.19</v>
+        <v>333897.64</v>
       </c>
     </row>
     <row r="57">
@@ -2234,16 +2234,16 @@
         </is>
       </c>
       <c r="F57" s="5" t="n">
-        <v>3.82</v>
+        <v>31.57</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>8640326</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>2261865.45</v>
+        <v>273687.87</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>2759475.84</v>
+        <v>333899.2</v>
       </c>
     </row>
     <row r="58">
@@ -2269,16 +2269,16 @@
         </is>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0.06</v>
+        <v>0.497</v>
       </c>
       <c r="G58" s="4" t="n">
         <v>116683.7</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>1944728.33</v>
+        <v>234776.06</v>
       </c>
       <c r="I58" s="4" t="n">
-        <v>2372568.57</v>
+        <v>286426.79</v>
       </c>
     </row>
     <row r="59">
@@ -2304,16 +2304,16 @@
         </is>
       </c>
       <c r="F59" s="5" t="n">
-        <v>2.178</v>
+        <v>18.004</v>
       </c>
       <c r="G59" s="4" t="n">
         <v>3869197</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>1776490.82</v>
+        <v>214907.63</v>
       </c>
       <c r="I59" s="4" t="n">
-        <v>2167318.8</v>
+        <v>262187.31</v>
       </c>
     </row>
     <row r="60">
@@ -2339,16 +2339,16 @@
         </is>
       </c>
       <c r="F60" s="5" t="n">
-        <v>0.081</v>
+        <v>0.67</v>
       </c>
       <c r="G60" s="4" t="n">
         <v>160404</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>1980296.3</v>
+        <v>239408.96</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>2415961.48</v>
+        <v>292078.93</v>
       </c>
     </row>
     <row r="61">
@@ -2693,16 +2693,16 @@
         </is>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0.056</v>
+        <v>0.466</v>
       </c>
       <c r="G72" s="4" t="n">
         <v>277081.2</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>4947878.57</v>
+        <v>594594.85</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>6036411.86</v>
+        <v>725405.72</v>
       </c>
     </row>
     <row r="73">
@@ -2728,16 +2728,16 @@
         </is>
       </c>
       <c r="F73" s="5" t="n">
-        <v>0.368</v>
+        <v>3.044</v>
       </c>
       <c r="G73" s="4" t="n">
         <v>1461797.94</v>
       </c>
       <c r="H73" s="4" t="n">
-        <v>3972277.01</v>
+        <v>480222.71</v>
       </c>
       <c r="I73" s="4" t="n">
-        <v>4846177.95</v>
+        <v>585871.71</v>
       </c>
     </row>
     <row r="74">
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="F74" s="8" t="n">
-        <v>43.283</v>
+        <v>357.704</v>
       </c>
       <c r="G74" s="9" t="n">
         <v>119899308.87</v>

</xml_diff>